<commit_message>
Groups and links from the platform structure; the Excel header as the questionnaire (v0.7, step 4, D-044, D-045)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/exemples/bases-fictives/travail-t1_surveymonkey.xlsx
+++ b/exemples/bases-fictives/travail-t1_surveymonkey.xlsx
@@ -784,7 +784,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Jamais</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -794,7 +794,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -814,7 +814,7 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -952,7 +952,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Toujours</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -962,7 +962,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -982,7 +982,7 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -1283,37 +1283,37 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
+          <t>Rarement</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Jamais</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Jamais</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Rarement</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
           <t>Toujours</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="R6" t="inlineStr">
         <is>
           <t>Jamais</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>Toujours</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>Rarement</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>Toujours</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr">
+      <c r="S6" t="inlineStr">
         <is>
           <t>Jamais</t>
-        </is>
-      </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>Toujours</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Toujours</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1466,7 +1466,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -1486,7 +1486,7 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
@@ -1634,7 +1634,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1664,7 +1664,7 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
@@ -1802,7 +1802,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Jamais</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1812,7 +1812,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
@@ -1832,7 +1832,7 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
@@ -1950,7 +1950,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1960,7 +1960,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Jamais</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
@@ -1980,7 +1980,7 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -2123,7 +2123,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -2133,7 +2133,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
@@ -2153,7 +2153,7 @@
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
@@ -2291,7 +2291,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Toujours</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -2301,7 +2301,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Toujours</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
@@ -2321,7 +2321,7 @@
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Jamais</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
@@ -2454,29 +2454,29 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
+          <t>Parfois</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Jamais</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>Jamais</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>Rarement</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
           <t>Toujours</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>Jamais</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>Parfois</t>
-        </is>
-      </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>Rarement</t>
-        </is>
-      </c>
-      <c r="Q13" t="inlineStr">
-        <is>
-          <t>Toujours</t>
-        </is>
-      </c>
       <c r="R13" t="inlineStr">
         <is>
           <t>Parfois</t>
@@ -2484,7 +2484,7 @@
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>Toujours</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
@@ -2617,37 +2617,37 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
+          <t>Toujours</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Toujours</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>Toujours</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>Toujours</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
           <t>Jamais</t>
         </is>
       </c>
-      <c r="N14" t="inlineStr">
+      <c r="R14" t="inlineStr">
         <is>
           <t>Toujours</t>
         </is>
       </c>
-      <c r="O14" t="inlineStr">
-        <is>
-          <t>Rarement</t>
-        </is>
-      </c>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t>Toujours</t>
-        </is>
-      </c>
-      <c r="Q14" t="inlineStr">
-        <is>
-          <t>Jamais</t>
-        </is>
-      </c>
-      <c r="R14" t="inlineStr">
-        <is>
-          <t>Toujours</t>
-        </is>
-      </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>Jamais</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
@@ -2810,7 +2810,7 @@
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
@@ -2953,7 +2953,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -2963,7 +2963,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
@@ -2983,7 +2983,7 @@
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
@@ -3121,7 +3121,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>Toujours</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -3131,7 +3131,7 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
@@ -3151,7 +3151,7 @@
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>Toujours</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
@@ -3279,7 +3279,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Jamais</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -3289,19 +3289,19 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
+          <t>Parfois</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>Rarement</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
           <t>Toujours</t>
         </is>
       </c>
-      <c r="P18" t="inlineStr">
-        <is>
-          <t>Rarement</t>
-        </is>
-      </c>
-      <c r="Q18" t="inlineStr">
-        <is>
-          <t>Toujours</t>
-        </is>
-      </c>
       <c r="R18" t="inlineStr">
         <is>
           <t>Jamais</t>
@@ -3309,7 +3309,7 @@
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Jamais</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
@@ -3442,37 +3442,37 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
+          <t>Jamais</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>Jamais</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>Jamais</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>Jamais</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
           <t>Toujours</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr">
+      <c r="R19" t="inlineStr">
         <is>
           <t>Jamais</t>
         </is>
       </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>Toujours</t>
-        </is>
-      </c>
-      <c r="P19" t="inlineStr">
+      <c r="S19" t="inlineStr">
         <is>
           <t>Jamais</t>
-        </is>
-      </c>
-      <c r="Q19" t="inlineStr">
-        <is>
-          <t>Toujours</t>
-        </is>
-      </c>
-      <c r="R19" t="inlineStr">
-        <is>
-          <t>Jamais</t>
-        </is>
-      </c>
-      <c r="S19" t="inlineStr">
-        <is>
-          <t>Souvent</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
@@ -3635,7 +3635,7 @@
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
@@ -3793,7 +3793,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -3803,7 +3803,7 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
@@ -3823,7 +3823,7 @@
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
@@ -3951,7 +3951,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Toujours</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -3961,27 +3961,27 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
+          <t>Toujours</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>Toujours</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
           <t>Jamais</t>
         </is>
       </c>
-      <c r="P22" t="inlineStr">
+      <c r="R22" t="inlineStr">
         <is>
           <t>Toujours</t>
         </is>
       </c>
-      <c r="Q22" t="inlineStr">
-        <is>
-          <t>Jamais</t>
-        </is>
-      </c>
-      <c r="R22" t="inlineStr">
+      <c r="S22" t="inlineStr">
         <is>
           <t>Toujours</t>
-        </is>
-      </c>
-      <c r="S22" t="inlineStr">
-        <is>
-          <t>Jamais</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
@@ -4267,7 +4267,7 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Jamais</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -4277,7 +4277,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Jamais</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
@@ -4297,7 +4297,7 @@
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
@@ -4420,7 +4420,7 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -4430,7 +4430,7 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
@@ -4450,7 +4450,7 @@
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
@@ -4583,37 +4583,37 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
+          <t>Souvent</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>Souvent</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>Toujours</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>Toujours</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
           <t>Jamais</t>
         </is>
       </c>
-      <c r="N26" t="inlineStr">
-        <is>
-          <t>Souvent</t>
-        </is>
-      </c>
-      <c r="O26" t="inlineStr">
-        <is>
-          <t>Rarement</t>
-        </is>
-      </c>
-      <c r="P26" t="inlineStr">
+      <c r="R26" t="inlineStr">
         <is>
           <t>Toujours</t>
         </is>
       </c>
-      <c r="Q26" t="inlineStr">
-        <is>
-          <t>Jamais</t>
-        </is>
-      </c>
-      <c r="R26" t="inlineStr">
+      <c r="S26" t="inlineStr">
         <is>
           <t>Toujours</t>
-        </is>
-      </c>
-      <c r="S26" t="inlineStr">
-        <is>
-          <t>Jamais</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
@@ -4751,7 +4751,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -4761,7 +4761,7 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Jamais</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
@@ -4781,7 +4781,7 @@
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>Toujours</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="T27" t="inlineStr">
@@ -5087,7 +5087,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -5117,7 +5117,7 @@
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="T29" t="inlineStr">
@@ -5285,7 +5285,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -5295,7 +5295,7 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
@@ -5315,7 +5315,7 @@
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
@@ -5621,29 +5621,29 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
+          <t>Rarement</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>Parfois</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>Parfois</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>Parfois</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
           <t>Jamais</t>
         </is>
       </c>
-      <c r="N32" t="inlineStr">
-        <is>
-          <t>Parfois</t>
-        </is>
-      </c>
-      <c r="O32" t="inlineStr">
-        <is>
-          <t>Rarement</t>
-        </is>
-      </c>
-      <c r="P32" t="inlineStr">
-        <is>
-          <t>Parfois</t>
-        </is>
-      </c>
-      <c r="Q32" t="inlineStr">
-        <is>
-          <t>Jamais</t>
-        </is>
-      </c>
       <c r="R32" t="inlineStr">
         <is>
           <t>Souvent</t>
@@ -5651,7 +5651,7 @@
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="T32" t="inlineStr">
@@ -5789,7 +5789,7 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
@@ -5799,7 +5799,7 @@
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
@@ -5819,7 +5819,7 @@
       </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="T33" t="inlineStr">
@@ -5972,7 +5972,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
@@ -5982,7 +5982,7 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
@@ -6002,7 +6002,7 @@
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>Jamais</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
@@ -6170,7 +6170,7 @@
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="T35" t="inlineStr">
@@ -6303,7 +6303,7 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>Jamais</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
@@ -6313,7 +6313,7 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="P36" t="inlineStr">
@@ -6481,7 +6481,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>Toujours</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -6491,7 +6491,7 @@
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>Toujours</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="P37" t="inlineStr">
@@ -6511,7 +6511,7 @@
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>Toujours</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="T37" t="inlineStr">
@@ -6654,7 +6654,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -6664,7 +6664,7 @@
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="P38" t="inlineStr">
@@ -6684,7 +6684,7 @@
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="T38" t="inlineStr">
@@ -6877,7 +6877,7 @@
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="T39" t="inlineStr">
@@ -7020,7 +7020,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -7030,7 +7030,7 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Jamais</t>
         </is>
       </c>
       <c r="P40" t="inlineStr">
@@ -7050,7 +7050,7 @@
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Jamais</t>
         </is>
       </c>
       <c r="T40" t="inlineStr">
@@ -7173,7 +7173,7 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
@@ -7183,7 +7183,7 @@
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="P41" t="inlineStr">
@@ -7203,7 +7203,7 @@
       </c>
       <c r="S41" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="T41" t="inlineStr">
@@ -7346,7 +7346,7 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Toujours</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
@@ -7356,7 +7356,7 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>Jamais</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="P42" t="inlineStr">
@@ -7376,7 +7376,7 @@
       </c>
       <c r="S42" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="T42" t="inlineStr">
@@ -7682,7 +7682,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
@@ -7692,7 +7692,7 @@
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="P44" t="inlineStr">
@@ -7712,7 +7712,7 @@
       </c>
       <c r="S44" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="T44" t="inlineStr">
@@ -7855,7 +7855,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>Toujours</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -7865,7 +7865,7 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="P45" t="inlineStr">
@@ -7885,7 +7885,7 @@
       </c>
       <c r="S45" t="inlineStr">
         <is>
-          <t>Toujours</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="T45" t="inlineStr">
@@ -8028,7 +8028,7 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>Jamais</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
@@ -8038,7 +8038,7 @@
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="P46" t="inlineStr">
@@ -8058,7 +8058,7 @@
       </c>
       <c r="S46" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="T46" t="inlineStr">
@@ -8196,7 +8196,7 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
@@ -8206,7 +8206,7 @@
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>Jamais</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="P47" t="inlineStr">
@@ -8226,7 +8226,7 @@
       </c>
       <c r="S47" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="T47" t="inlineStr">
@@ -8379,7 +8379,7 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
@@ -8389,7 +8389,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Jamais</t>
         </is>
       </c>
       <c r="P48" t="inlineStr">
@@ -8409,7 +8409,7 @@
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>Toujours</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="T48" t="inlineStr">
@@ -8537,37 +8537,37 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
+          <t>Jamais</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>Rarement</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>Rarement</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>Jamais</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
           <t>Toujours</t>
         </is>
       </c>
-      <c r="N49" t="inlineStr">
-        <is>
-          <t>Rarement</t>
-        </is>
-      </c>
-      <c r="O49" t="inlineStr">
-        <is>
-          <t>Toujours</t>
-        </is>
-      </c>
-      <c r="P49" t="inlineStr">
+      <c r="R49" t="inlineStr">
         <is>
           <t>Jamais</t>
         </is>
       </c>
-      <c r="Q49" t="inlineStr">
-        <is>
-          <t>Toujours</t>
-        </is>
-      </c>
-      <c r="R49" t="inlineStr">
-        <is>
-          <t>Jamais</t>
-        </is>
-      </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>Toujours</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="T49" t="inlineStr">
@@ -8705,29 +8705,29 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
+          <t>Parfois</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>Jamais</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>Rarement</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>Jamais</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
           <t>Toujours</t>
         </is>
       </c>
-      <c r="N50" t="inlineStr">
-        <is>
-          <t>Jamais</t>
-        </is>
-      </c>
-      <c r="O50" t="inlineStr">
-        <is>
-          <t>Souvent</t>
-        </is>
-      </c>
-      <c r="P50" t="inlineStr">
-        <is>
-          <t>Jamais</t>
-        </is>
-      </c>
-      <c r="Q50" t="inlineStr">
-        <is>
-          <t>Toujours</t>
-        </is>
-      </c>
       <c r="R50" t="inlineStr">
         <is>
           <t>Rarement</t>
@@ -8735,7 +8735,7 @@
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t>Toujours</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="T50" t="inlineStr">
@@ -9041,37 +9041,37 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
+          <t>Toujours</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>Toujours</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>Souvent</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>Toujours</t>
+        </is>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
           <t>Jamais</t>
         </is>
       </c>
-      <c r="N52" t="inlineStr">
+      <c r="R52" t="inlineStr">
         <is>
           <t>Toujours</t>
         </is>
       </c>
-      <c r="O52" t="inlineStr">
-        <is>
-          <t>Jamais</t>
-        </is>
-      </c>
-      <c r="P52" t="inlineStr">
+      <c r="S52" t="inlineStr">
         <is>
           <t>Toujours</t>
-        </is>
-      </c>
-      <c r="Q52" t="inlineStr">
-        <is>
-          <t>Jamais</t>
-        </is>
-      </c>
-      <c r="R52" t="inlineStr">
-        <is>
-          <t>Toujours</t>
-        </is>
-      </c>
-      <c r="S52" t="inlineStr">
-        <is>
-          <t>Parfois</t>
         </is>
       </c>
       <c r="T52" t="inlineStr">
@@ -9209,7 +9209,7 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Toujours</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
@@ -9219,7 +9219,7 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Toujours</t>
         </is>
       </c>
       <c r="P53" t="inlineStr">
@@ -9239,7 +9239,7 @@
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="T53" t="inlineStr">
@@ -9367,7 +9367,7 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
@@ -9377,7 +9377,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="P54" t="inlineStr">
@@ -9397,7 +9397,7 @@
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="T54" t="inlineStr">
@@ -9545,7 +9545,7 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>Jamais</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="N55" t="inlineStr">
@@ -9555,7 +9555,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>Jamais</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="P55" t="inlineStr">
@@ -9575,7 +9575,7 @@
       </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t>Jamais</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="T55" t="inlineStr">
@@ -9728,7 +9728,7 @@
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="P56" t="inlineStr">
@@ -9748,7 +9748,7 @@
       </c>
       <c r="S56" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="T56" t="inlineStr">
@@ -9886,7 +9886,7 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="N57" t="inlineStr">
@@ -9896,7 +9896,7 @@
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="P57" t="inlineStr">
@@ -10054,7 +10054,7 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="N58" t="inlineStr">
@@ -10084,7 +10084,7 @@
       </c>
       <c r="S58" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="T58" t="inlineStr">
@@ -10272,7 +10272,7 @@
       </c>
       <c r="S59" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="T59" t="inlineStr">
@@ -10761,7 +10761,7 @@
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="N62" t="inlineStr">
@@ -10771,7 +10771,7 @@
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="P62" t="inlineStr">
@@ -10791,7 +10791,7 @@
       </c>
       <c r="S62" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="T62" t="inlineStr">
@@ -10939,7 +10939,7 @@
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="N63" t="inlineStr">
@@ -10949,7 +10949,7 @@
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>Jamais</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="P63" t="inlineStr">
@@ -10969,7 +10969,7 @@
       </c>
       <c r="S63" t="inlineStr">
         <is>
-          <t>Jamais</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="T63" t="inlineStr">
@@ -11092,7 +11092,7 @@
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>Jamais</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="N64" t="inlineStr">
@@ -11102,7 +11102,7 @@
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>Jamais</t>
+          <t>Toujours</t>
         </is>
       </c>
       <c r="P64" t="inlineStr">
@@ -11122,7 +11122,7 @@
       </c>
       <c r="S64" t="inlineStr">
         <is>
-          <t>Jamais</t>
+          <t>Toujours</t>
         </is>
       </c>
       <c r="T64" t="inlineStr">
@@ -11240,7 +11240,7 @@
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="N65" t="inlineStr">
@@ -11250,7 +11250,7 @@
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="P65" t="inlineStr">
@@ -11270,7 +11270,7 @@
       </c>
       <c r="S65" t="inlineStr">
         <is>
-          <t>Jamais</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="T65" t="inlineStr">
@@ -11438,7 +11438,7 @@
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>Jamais</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="N66" t="inlineStr">
@@ -11448,7 +11448,7 @@
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="P66" t="inlineStr">
@@ -11468,7 +11468,7 @@
       </c>
       <c r="S66" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Toujours</t>
         </is>
       </c>
       <c r="T66" t="inlineStr">
@@ -11779,7 +11779,7 @@
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="N68" t="inlineStr">
@@ -11789,7 +11789,7 @@
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="P68" t="inlineStr">
@@ -11809,7 +11809,7 @@
       </c>
       <c r="S68" t="inlineStr">
         <is>
-          <t>Jamais</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="T68" t="inlineStr">
@@ -11962,7 +11962,7 @@
       </c>
       <c r="S69" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="T69" t="inlineStr">
@@ -12090,7 +12090,7 @@
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Jamais</t>
         </is>
       </c>
       <c r="N70" t="inlineStr">
@@ -12100,7 +12100,7 @@
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Jamais</t>
         </is>
       </c>
       <c r="P70" t="inlineStr">
@@ -12120,7 +12120,7 @@
       </c>
       <c r="S70" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Jamais</t>
         </is>
       </c>
       <c r="T70" t="inlineStr">
@@ -12243,29 +12243,29 @@
       </c>
       <c r="M71" t="inlineStr">
         <is>
+          <t>Souvent</t>
+        </is>
+      </c>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>Souvent</t>
+        </is>
+      </c>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>Jamais</t>
+        </is>
+      </c>
+      <c r="P71" t="inlineStr">
+        <is>
+          <t>Parfois</t>
+        </is>
+      </c>
+      <c r="Q71" t="inlineStr">
+        <is>
           <t>Toujours</t>
         </is>
       </c>
-      <c r="N71" t="inlineStr">
-        <is>
-          <t>Souvent</t>
-        </is>
-      </c>
-      <c r="O71" t="inlineStr">
-        <is>
-          <t>Parfois</t>
-        </is>
-      </c>
-      <c r="P71" t="inlineStr">
-        <is>
-          <t>Parfois</t>
-        </is>
-      </c>
-      <c r="Q71" t="inlineStr">
-        <is>
-          <t>Toujours</t>
-        </is>
-      </c>
       <c r="R71" t="inlineStr">
         <is>
           <t>Rarement</t>
@@ -12273,7 +12273,7 @@
       </c>
       <c r="S71" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="T71" t="inlineStr">
@@ -12411,7 +12411,7 @@
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="N72" t="inlineStr">
@@ -12579,7 +12579,7 @@
       </c>
       <c r="M73" t="inlineStr">
         <is>
-          <t>Toujours</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="N73" t="inlineStr">
@@ -12589,7 +12589,7 @@
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>Toujours</t>
+          <t>Jamais</t>
         </is>
       </c>
       <c r="P73" t="inlineStr">
@@ -12609,7 +12609,7 @@
       </c>
       <c r="S73" t="inlineStr">
         <is>
-          <t>Toujours</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="T73" t="inlineStr">
@@ -12752,7 +12752,7 @@
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="P74" t="inlineStr">
@@ -12900,7 +12900,7 @@
       </c>
       <c r="M75" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="N75" t="inlineStr">
@@ -12910,7 +12910,7 @@
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="P75" t="inlineStr">
@@ -12930,7 +12930,7 @@
       </c>
       <c r="S75" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="T75" t="inlineStr">
@@ -13063,7 +13063,7 @@
       </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="N76" t="inlineStr">
@@ -13073,7 +13073,7 @@
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>Toujours</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="P76" t="inlineStr">
@@ -13093,7 +13093,7 @@
       </c>
       <c r="S76" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="T76" t="inlineStr">
@@ -13226,7 +13226,7 @@
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Jamais</t>
         </is>
       </c>
       <c r="N77" t="inlineStr">
@@ -13236,7 +13236,7 @@
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="P77" t="inlineStr">
@@ -13256,7 +13256,7 @@
       </c>
       <c r="S77" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Jamais</t>
         </is>
       </c>
       <c r="T77" t="inlineStr">
@@ -13389,7 +13389,7 @@
       </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Toujours</t>
         </is>
       </c>
       <c r="N78" t="inlineStr">
@@ -13399,7 +13399,7 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Toujours</t>
         </is>
       </c>
       <c r="P78" t="inlineStr">
@@ -13419,7 +13419,7 @@
       </c>
       <c r="S78" t="inlineStr">
         <is>
-          <t>Jamais</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="T78" t="inlineStr">
@@ -13557,7 +13557,7 @@
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="N79" t="inlineStr">
@@ -13567,7 +13567,7 @@
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="P79" t="inlineStr">
@@ -13587,7 +13587,7 @@
       </c>
       <c r="S79" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="T79" t="inlineStr">
@@ -13908,7 +13908,7 @@
       </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t>Toujours</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="N81" t="inlineStr">
@@ -13938,7 +13938,7 @@
       </c>
       <c r="S81" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="T81" t="inlineStr">
@@ -14071,7 +14071,7 @@
       </c>
       <c r="M82" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="N82" t="inlineStr">
@@ -14081,7 +14081,7 @@
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t>Jamais</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="P82" t="inlineStr">
@@ -14101,7 +14101,7 @@
       </c>
       <c r="S82" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="T82" t="inlineStr">
@@ -14239,7 +14239,7 @@
       </c>
       <c r="M83" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="N83" t="inlineStr">
@@ -14249,7 +14249,7 @@
       </c>
       <c r="O83" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Toujours</t>
         </is>
       </c>
       <c r="P83" t="inlineStr">
@@ -14269,7 +14269,7 @@
       </c>
       <c r="S83" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="T83" t="inlineStr">
@@ -14570,7 +14570,7 @@
       </c>
       <c r="M85" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="N85" t="inlineStr">
@@ -14580,7 +14580,7 @@
       </c>
       <c r="O85" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="P85" t="inlineStr">
@@ -14600,7 +14600,7 @@
       </c>
       <c r="S85" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="T85" t="inlineStr">
@@ -14738,7 +14738,7 @@
       </c>
       <c r="M86" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="N86" t="inlineStr">
@@ -14748,7 +14748,7 @@
       </c>
       <c r="O86" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="P86" t="inlineStr">
@@ -14768,7 +14768,7 @@
       </c>
       <c r="S86" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="T86" t="inlineStr">
@@ -14886,7 +14886,7 @@
       </c>
       <c r="M87" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="N87" t="inlineStr">
@@ -14896,7 +14896,7 @@
       </c>
       <c r="O87" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="P87" t="inlineStr">
@@ -14916,7 +14916,7 @@
       </c>
       <c r="S87" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="T87" t="inlineStr">
@@ -15054,7 +15054,7 @@
       </c>
       <c r="M88" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="N88" t="inlineStr">
@@ -15084,7 +15084,7 @@
       </c>
       <c r="S88" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="T88" t="inlineStr">
@@ -15227,7 +15227,7 @@
       </c>
       <c r="M89" t="inlineStr">
         <is>
-          <t>Toujours</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="N89" t="inlineStr">
@@ -15237,7 +15237,7 @@
       </c>
       <c r="O89" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="P89" t="inlineStr">
@@ -15257,7 +15257,7 @@
       </c>
       <c r="S89" t="inlineStr">
         <is>
-          <t>Toujours</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="T89" t="inlineStr">
@@ -15405,7 +15405,7 @@
       </c>
       <c r="M90" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="N90" t="inlineStr">
@@ -15415,7 +15415,7 @@
       </c>
       <c r="O90" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="P90" t="inlineStr">
@@ -15435,7 +15435,7 @@
       </c>
       <c r="S90" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="T90" t="inlineStr">
@@ -15573,7 +15573,7 @@
       </c>
       <c r="M91" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="N91" t="inlineStr">
@@ -15603,7 +15603,7 @@
       </c>
       <c r="S91" t="inlineStr">
         <is>
-          <t>Jamais</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="T91" t="inlineStr">
@@ -15741,7 +15741,7 @@
       </c>
       <c r="M92" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="N92" t="inlineStr">
@@ -15751,7 +15751,7 @@
       </c>
       <c r="O92" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="P92" t="inlineStr">
@@ -15771,7 +15771,7 @@
       </c>
       <c r="S92" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="T92" t="inlineStr">
@@ -15914,7 +15914,7 @@
       </c>
       <c r="M93" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="N93" t="inlineStr">
@@ -15924,7 +15924,7 @@
       </c>
       <c r="O93" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="P93" t="inlineStr">
@@ -15944,7 +15944,7 @@
       </c>
       <c r="S93" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="T93" t="inlineStr">
@@ -16280,7 +16280,7 @@
       </c>
       <c r="M95" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="N95" t="inlineStr">
@@ -16290,7 +16290,7 @@
       </c>
       <c r="O95" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Toujours</t>
         </is>
       </c>
       <c r="P95" t="inlineStr">
@@ -16310,7 +16310,7 @@
       </c>
       <c r="S95" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="T95" t="inlineStr">
@@ -16438,7 +16438,7 @@
       </c>
       <c r="M96" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="N96" t="inlineStr">
@@ -16621,7 +16621,7 @@
       </c>
       <c r="M97" t="inlineStr">
         <is>
-          <t>Jamais</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="N97" t="inlineStr">
@@ -16631,7 +16631,7 @@
       </c>
       <c r="O97" t="inlineStr">
         <is>
-          <t>Jamais</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="P97" t="inlineStr">
@@ -16651,7 +16651,7 @@
       </c>
       <c r="S97" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Toujours</t>
         </is>
       </c>
       <c r="T97" t="inlineStr">
@@ -16774,7 +16774,7 @@
       </c>
       <c r="M98" t="inlineStr">
         <is>
-          <t>Jamais</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="N98" t="inlineStr">
@@ -16784,7 +16784,7 @@
       </c>
       <c r="O98" t="inlineStr">
         <is>
-          <t>Jamais</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="P98" t="inlineStr">
@@ -16804,7 +16804,7 @@
       </c>
       <c r="S98" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Toujours</t>
         </is>
       </c>
       <c r="T98" t="inlineStr">
@@ -16952,7 +16952,7 @@
       </c>
       <c r="M99" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="N99" t="inlineStr">
@@ -16962,7 +16962,7 @@
       </c>
       <c r="O99" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="P99" t="inlineStr">
@@ -16982,7 +16982,7 @@
       </c>
       <c r="S99" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="T99" t="inlineStr">
@@ -17105,7 +17105,7 @@
       </c>
       <c r="M100" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="N100" t="inlineStr">
@@ -17115,7 +17115,7 @@
       </c>
       <c r="O100" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="P100" t="inlineStr">
@@ -17135,7 +17135,7 @@
       </c>
       <c r="S100" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="T100" t="inlineStr">
@@ -17441,7 +17441,7 @@
       </c>
       <c r="M102" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Jamais</t>
         </is>
       </c>
       <c r="N102" t="inlineStr">
@@ -17614,7 +17614,7 @@
       </c>
       <c r="M103" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Jamais</t>
         </is>
       </c>
       <c r="N103" t="inlineStr">
@@ -17624,7 +17624,7 @@
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="P103" t="inlineStr">
@@ -17644,7 +17644,7 @@
       </c>
       <c r="S103" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Jamais</t>
         </is>
       </c>
       <c r="T103" t="inlineStr">
@@ -17777,7 +17777,7 @@
       </c>
       <c r="M104" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="N104" t="inlineStr">
@@ -17787,7 +17787,7 @@
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="P104" t="inlineStr">
@@ -17807,7 +17807,7 @@
       </c>
       <c r="S104" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="T104" t="inlineStr">
@@ -17940,7 +17940,7 @@
       </c>
       <c r="M105" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="N105" t="inlineStr">
@@ -17950,7 +17950,7 @@
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="P105" t="inlineStr">
@@ -17970,7 +17970,7 @@
       </c>
       <c r="S105" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="T105" t="inlineStr">
@@ -18108,7 +18108,7 @@
       </c>
       <c r="O106" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="P106" t="inlineStr">
@@ -18459,7 +18459,7 @@
       </c>
       <c r="S108" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="T108" t="inlineStr">
@@ -18582,7 +18582,7 @@
       </c>
       <c r="M109" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Toujours</t>
         </is>
       </c>
       <c r="N109" t="inlineStr">
@@ -18592,7 +18592,7 @@
       </c>
       <c r="O109" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="P109" t="inlineStr">
@@ -18612,7 +18612,7 @@
       </c>
       <c r="S109" t="inlineStr">
         <is>
-          <t>Jamais</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="T109" t="inlineStr">
@@ -18735,7 +18735,7 @@
       </c>
       <c r="M110" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="N110" t="inlineStr">
@@ -18745,7 +18745,7 @@
       </c>
       <c r="O110" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="P110" t="inlineStr">
@@ -18765,7 +18765,7 @@
       </c>
       <c r="S110" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="T110" t="inlineStr">
@@ -18918,7 +18918,7 @@
       </c>
       <c r="M111" t="inlineStr">
         <is>
-          <t>Toujours</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="N111" t="inlineStr">
@@ -18928,7 +18928,7 @@
       </c>
       <c r="O111" t="inlineStr">
         <is>
-          <t>Toujours</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="P111" t="inlineStr">
@@ -18948,7 +18948,7 @@
       </c>
       <c r="S111" t="inlineStr">
         <is>
-          <t>Toujours</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="T111" t="inlineStr">
@@ -19091,7 +19091,7 @@
       </c>
       <c r="M112" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Toujours</t>
         </is>
       </c>
       <c r="N112" t="inlineStr">
@@ -19101,7 +19101,7 @@
       </c>
       <c r="O112" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Toujours</t>
         </is>
       </c>
       <c r="P112" t="inlineStr">
@@ -19121,7 +19121,7 @@
       </c>
       <c r="S112" t="inlineStr">
         <is>
-          <t>Jamais</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="T112" t="inlineStr">
@@ -19259,7 +19259,7 @@
       </c>
       <c r="M113" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="N113" t="inlineStr">
@@ -19269,7 +19269,7 @@
       </c>
       <c r="O113" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="P113" t="inlineStr">
@@ -19289,7 +19289,7 @@
       </c>
       <c r="S113" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="T113" t="inlineStr">
@@ -19432,7 +19432,7 @@
       </c>
       <c r="M114" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="N114" t="inlineStr">
@@ -19442,7 +19442,7 @@
       </c>
       <c r="O114" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Toujours</t>
         </is>
       </c>
       <c r="P114" t="inlineStr">
@@ -19462,7 +19462,7 @@
       </c>
       <c r="S114" t="inlineStr">
         <is>
-          <t>Jamais</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="T114" t="inlineStr">
@@ -19610,7 +19610,7 @@
       </c>
       <c r="M115" t="inlineStr">
         <is>
-          <t>Jamais</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="N115" t="inlineStr">
@@ -19620,7 +19620,7 @@
       </c>
       <c r="O115" t="inlineStr">
         <is>
-          <t>Jamais</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="P115" t="inlineStr">
@@ -19640,7 +19640,7 @@
       </c>
       <c r="S115" t="inlineStr">
         <is>
-          <t>Jamais</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="T115" t="inlineStr">
@@ -19788,7 +19788,7 @@
       </c>
       <c r="M116" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Jamais</t>
         </is>
       </c>
       <c r="N116" t="inlineStr">
@@ -19798,7 +19798,7 @@
       </c>
       <c r="O116" t="inlineStr">
         <is>
-          <t>Toujours</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="P116" t="inlineStr">
@@ -19818,7 +19818,7 @@
       </c>
       <c r="S116" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Jamais</t>
         </is>
       </c>
       <c r="T116" t="inlineStr">
@@ -19936,7 +19936,7 @@
       </c>
       <c r="M117" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="N117" t="inlineStr">
@@ -19946,7 +19946,7 @@
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="P117" t="inlineStr">
@@ -19966,7 +19966,7 @@
       </c>
       <c r="S117" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Jamais</t>
         </is>
       </c>
       <c r="T117" t="inlineStr">
@@ -20104,7 +20104,7 @@
       </c>
       <c r="M118" t="inlineStr">
         <is>
-          <t>Toujours</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="N118" t="inlineStr">
@@ -20114,7 +20114,7 @@
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>Toujours</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="P118" t="inlineStr">
@@ -20134,7 +20134,7 @@
       </c>
       <c r="S118" t="inlineStr">
         <is>
-          <t>Toujours</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="T118" t="inlineStr">
@@ -20267,7 +20267,7 @@
       </c>
       <c r="M119" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Jamais</t>
         </is>
       </c>
       <c r="N119" t="inlineStr">
@@ -20277,7 +20277,7 @@
       </c>
       <c r="O119" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Jamais</t>
         </is>
       </c>
       <c r="P119" t="inlineStr">
@@ -20297,7 +20297,7 @@
       </c>
       <c r="S119" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Jamais</t>
         </is>
       </c>
       <c r="T119" t="inlineStr">
@@ -20450,7 +20450,7 @@
       </c>
       <c r="M120" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Parfois</t>
         </is>
       </c>
       <c r="N120" t="inlineStr">
@@ -20460,7 +20460,7 @@
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="P120" t="inlineStr">
@@ -20480,7 +20480,7 @@
       </c>
       <c r="S120" t="inlineStr">
         <is>
-          <t>Rarement</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="T120" t="inlineStr">
@@ -20648,7 +20648,7 @@
       </c>
       <c r="S121" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Souvent</t>
         </is>
       </c>
       <c r="T121" t="inlineStr">
@@ -20786,7 +20786,7 @@
       </c>
       <c r="M122" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="N122" t="inlineStr">
@@ -20796,7 +20796,7 @@
       </c>
       <c r="O122" t="inlineStr">
         <is>
-          <t>Souvent</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="P122" t="inlineStr">
@@ -20816,7 +20816,7 @@
       </c>
       <c r="S122" t="inlineStr">
         <is>
-          <t>Parfois</t>
+          <t>Rarement</t>
         </is>
       </c>
       <c r="T122" t="inlineStr">

</xml_diff>